<commit_message>
Modified XLSX Sheet 2
</commit_message>
<xml_diff>
--- a/Documents/Proje__Kontrol_Listesi_481.xlsx
+++ b/Documents/Proje__Kontrol_Listesi_481.xlsx
@@ -494,7 +494,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="162">
   <si>
     <t xml:space="preserve">Proje Grubu adi:</t>
   </si>
@@ -1185,6 +1185,9 @@
       </rPr>
       <t xml:space="preserve"> etc.</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Demo</t>
   </si>
   <si>
     <t xml:space="preserve">Statik sitelerin çalışırken çok düşük düzeyde sunucu işlem gücü gerektirmesi, harcanan enerjiyi ve karbon ayak izini minimize ederek iklim krizi ile mücadeleye pozitif yönde katkı sağlar.</t>
@@ -1298,6 +1301,9 @@
       </rPr>
       <t xml:space="preserve"> kurallara uygunluk sağlanmış mı? Ilgili yasal kurallara , standartlara ve etik ilkelere referans verilmis mi</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">LICENCE</t>
   </si>
   <si>
     <t xml:space="preserve">Projede kullanılan üçüncü parti açık kaynak kütüphanelerin lisanslarına (MIT, Apache vb.) tam uyum sağlandığı dokümante edilmiştir. Araç son kullanıcıdan dinamik veri toplamadığı için KVKK/GDPR gibi veri gizliliği yasalarıyla doğal olarak uyumludur.</t>
@@ -2325,10 +2331,10 @@
         <v>151</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>20</v>
+        <v>152</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>13</v>
@@ -2337,16 +2343,16 @@
     </row>
     <row r="38" customFormat="false" ht="44.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E38" s="9" t="s">
         <v>13</v>
@@ -2355,16 +2361,16 @@
     </row>
     <row r="39" customFormat="false" ht="44.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>20</v>
+        <v>160</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>13</v>

</xml_diff>